<commit_message>
Separate Basket 3 and refine September profiles
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -3893,7 +3893,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Hanging Basket 3</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3930,7 +3930,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Hanging Basket 3</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3967,7 +3967,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Hanging Basket 3</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4004,7 +4004,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Hanging Basket 3</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -4041,7 +4041,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Hanging Basket 3</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Improve all plant profiles and move new pots to Steps
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant Guide" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$182</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plant Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G180"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6303,32 +6303,32 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple' · Pot 1</t>
+          <t>Mixed Pot</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple'</t>
+          <t>Mixed seasonal planting — contents to confirm</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Bright outdoor position; confirm the needs of each constituent plant when identified.</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist and well drained while establishing.</t>
+          <t>Check the compost frequently in warm or windy weather; supplied by an adjustable sprinkler.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>Trim trails to shape and keep stems clear of the neighbouring Skimmia and Pansies.</t>
+          <t>Deadhead finished flowers, keep the drainage holes clear and record the individual plants and cultivars as labels or clearer photographs become available.</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Evergreen variegated foliage provides year-round structure.</t>
+          <t>A mixed seasonal container providing varied flower colour; exact contents remain unresolved.</t>
         </is>
       </c>
     </row>
@@ -6340,49 +6340,49 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Double Diamond'</t>
+          <t>Fuchsia Pot</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Double Diamond'</t>
+          <t>Fuchsia cultivars — identities to confirm</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to shade in a sheltered position.</t>
+          <t>Bright light or partial shade, protected from the harshest reflected afternoon heat.</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
+          <t>Keep the compost evenly moist but freely drained; supplied by an adjustable sprinkler.</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Use ericaceous compost, keep the crown clear and protect the pot from winter waterlogging.</t>
+          <t>Deadhead for continued flowering, check the sprinkler reaches the compost rather than only the foliage, and confirm whether the plants are hardy before winter.</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage gives structure; flower and berry details will be observed as the plant establishes.</t>
+          <t>Pendant Fuchsia flowers through summer and autumn; exact cultivars and winter hardiness remain unresolved.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>Stairs Pots</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Pansy 'Fire Red' · Pot 1</t>
+          <t>Hedera helix 'Yellow Ripple' · Pot 1</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Viola × wittrockiana 'Fire Red'</t>
+          <t>Hedera helix 'Yellow Ripple'</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -6392,108 +6392,108 @@
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist without saturation.</t>
+          <t>Keep compost evenly moist and well drained while establishing.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Remove faded flowers and seed pods to prolong the cool-season display.</t>
+          <t>Trim trails to shape and keep stems clear of the neighbouring Skimmia and Pansies.</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Red flowers provide autumn-to-spring container colour.</t>
+          <t>Evergreen variegated foliage provides year-round structure.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>Stairs Pots</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple' · Pot 2</t>
+          <t>Skimmia 'Double Diamond'</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple'</t>
+          <t>Skimmia 'Double Diamond'</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Partial shade to shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist and well drained while establishing.</t>
+          <t>Keep compost evenly moist and freely drained.</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>Trim trails to shape and keep stems clear of the Gaultheria and Pansies.</t>
+          <t>Use ordinary peat-free container compost, keep the crown clear and protect the pot from winter waterlogging.</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Evergreen variegated foliage provides year-round structure.</t>
+          <t>Evergreen foliage gives structure; flower and berry details will be observed as the plant establishes.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>Stairs Pots</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Gaultheria (cultivar to confirm)</t>
+          <t>Pansy 'Fire Red' · Pot 1</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Gaultheria — cultivar to confirm</t>
+          <t>Viola × wittrockiana 'Fire Red'</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to shade.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist and acidic, never waterlogged.</t>
+          <t>Keep compost evenly moist without saturation.</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>Use ericaceous compost and rainwater where possible. Retain a label or berry and foliage close-up before assigning a cultivar.</t>
+          <t>Remove faded flowers and seed pods to prolong the cool-season display.</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage and possible autumn berries; cultivar is not yet confirmed.</t>
+          <t>Red flowers provide autumn-to-spring container colour.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>Stairs Pots</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Pansy 'Fire Red' · Pot 2</t>
+          <t>Hedera helix 'Yellow Ripple' · Pot 2</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Viola × wittrockiana 'Fire Red'</t>
+          <t>Hedera helix 'Yellow Ripple'</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -6503,461 +6503,461 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist without saturation.</t>
+          <t>Keep compost evenly moist and well drained while establishing.</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>Remove faded flowers and seed pods to prolong the cool-season display.</t>
+          <t>Trim trails to shape and keep stems clear of the Gaultheria and Pansies.</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>Red flowers provide autumn-to-spring container colour.</t>
+          <t>Evergreen variegated foliage provides year-round structure.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Front Strawberry Tree</t>
+          <t>Stairs Pots</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Arbutus unedo</t>
+          <t>Gaultheria (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Arbutus unedo</t>
+          <t>Gaultheria — cultivar to confirm</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a sheltered, well-drained position.</t>
+          <t>Partial shade to shade.</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Water regularly through the first two years, increasing in hot or dry weather; avoid waterlogging.</t>
+          <t>Keep compost evenly moist and acidic, never waterlogged.</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>Keep a clear, mulched root area while it establishes. Prune only to remove damaged or crossing growth, and stake a young standard tree until secure.</t>
+          <t>Use ericaceous compost and rainwater where possible. Retain a label or berry and foliage close-up before assigning a cultivar.</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage; white urn-shaped autumn flowers and ornamental red fruits can appear together on established plants.</t>
+          <t>Evergreen foliage and possible autumn berries; cultivar is not yet confirmed.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Front Fruit Trees</t>
+          <t>Stairs Pots</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Apple Tree</t>
+          <t>Pansy 'Fire Red' · Pot 2</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Malus domestica</t>
+          <t>Viola × wittrockiana 'Fire Red'</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>Water well in dry spells while fruiting.</t>
+          <t>Keep compost evenly moist without saturation.</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>Winter prune for shape and airflow; thin fruit in June if heavy.</t>
+          <t>Remove faded flowers and seed pods to prolong the cool-season display.</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>Blossom April–May; fruit late summer–autumn.</t>
+          <t>Red flowers provide autumn-to-spring container colour.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Front Fruit Trees</t>
+          <t>Front Strawberry Tree</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Damson Tree</t>
+          <t>Arbutus unedo</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>Prunus domestica subsp. insititia (cultivar to confirm)</t>
+          <t>Arbutus unedo</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>Full sun for reliable blossom and fruit ripening.</t>
+          <t>Full sun in a sheltered, well-drained position.</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>Water deeply during prolonged dry spells, especially from fruit set to harvest.</t>
+          <t>Water regularly through the first two years, increasing in hot or dry weather; avoid waterlogging.</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>Prune only in dry summer weather to reduce silver-leaf and canker risk; remove suckers from below the graft.</t>
+          <t>Keep a clear, mulched root area while it establishes. Prune only to remove damaged or crossing growth, and stake a young standard tree until secure.</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>White spring blossom followed by blue-black damsons in late summer or early autumn.</t>
+          <t>Evergreen foliage; white urn-shaped autumn flowers and ornamental red fruits can appear together on established plants.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Front Gate Tree</t>
+          <t>Front Fruit Trees</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Weeping Crab Apple (cultivar to confirm)</t>
+          <t>Apple Tree</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Malus (weeping cultivar; 'Red Jade' is a best-fit possibility)</t>
+          <t>Malus domestica</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the best blossom, fruit colour and balanced growth.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Water deeply during prolonged drought, particularly while establishing and while fruit is swelling.</t>
+          <t>Water well in dry spells while fruiting.</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>Remove dead, damaged and crossing wood in winter, preserving the natural weeping framework. Record blossom and ripe-fruit details before naming the cultivar.</t>
+          <t>Winter prune for shape and airflow; thin fruit in June if heavy.</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>Spring blossom followed by small ornamental crab apples that can persist into autumn and winter.</t>
+          <t>Blossom April–May; fruit late summer–autumn.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>House · Hallway · Kentia Palm</t>
+          <t>Front Fruit Trees</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Kentia Palm — assumed</t>
+          <t>Damson Tree</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>Howea forsteriana</t>
+          <t>Prunus domestica subsp. insititia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect light; protect the fronds from strong direct sun.</t>
+          <t>Full sun for reliable blossom and fruit ripening.</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>Check the upper few centimetres of compost before watering, then drain fully and empty the white cachepot.</t>
+          <t>Water deeply during prolonged dry spells, especially from fruit set to harvest.</t>
         </is>
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>Maintain moderate humidity, keep away from cold draughts and radiators, and feed monthly during active spring and summer growth.</t>
+          <t>Prune only in dry summer weather to reduce silver-leaf and canker risk; remove suckers from below the graft.</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>Evergreen indoor foliage throughout the year; growth slows as light levels fall in winter.</t>
+          <t>White spring blossom followed by blue-black damsons in late summer or early autumn.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>House · Kitchen / Dining · ‘Gioia’ Fern</t>
+          <t>Front Gate Tree</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Bird’s Nest Fern ‘Gioia’</t>
+          <t>Weeping Crab Apple (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Asplenium antiquum ‘Gioia’</t>
+          <t>Malus (weeping cultivar; 'Red Jade' is a best-fit possibility)</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
+          <t>Full sun for the best blossom, fruit colour and balanced growth.</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
+          <t>Water deeply during prolonged drought, particularly while establishing and while fruit is swelling.</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
+          <t>Remove dead, damaged and crossing wood in winter, preserving the natural weeping framework. Record blossom and ripe-fruit details before naming the cultivar.</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
+          <t>Spring blossom followed by small ornamental crab apples that can persist into autumn and winter.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>House · Hallway · Staghorn Fern</t>
+          <t>House · Hallway · Kentia Palm</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Staghorn Fern</t>
+          <t>Kentia Palm — assumed</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Platycerium bifurcatum</t>
+          <t>Howea forsteriana</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
+          <t>Bright indirect light; protect the fronds from strong direct sun.</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
+          <t>Check the upper few centimetres of compost before watering, then drain fully and empty the white cachepot.</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
+          <t>Maintain moderate humidity, keep away from cold draughts and radiators, and feed monthly during active spring and summer growth.</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows as light levels fall in winter.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · Shared Pot · Spider Plant</t>
+          <t>House · Kitchen / Dining · ‘Gioia’ Fern</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Spider Plant ‘Vittatum’ — assumed</t>
+          <t>Bird’s Nest Fern ‘Gioia’</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Chlorophytum comosum ‘Vittatum’</t>
+          <t>Asplenium antiquum ‘Gioia’</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect light is ideal; it tolerates lower light but direct hot sun can scorch the striped leaves.</t>
+          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>Allow the compost surface to begin drying, then water thoroughly and let the shared container drain fully.</t>
+          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>Trim only spent stems or badly damaged leaves, feed lightly during active growth and root the hanging plantlets if wanted.</t>
+          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>Evergreen striped foliage and hanging plantlets are the year-round display; growth slows in winter.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · Shared Pot · Parlour Palm</t>
+          <t>House · Hallway · Staghorn Fern</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>Parlour Palm — assumed</t>
+          <t>Staghorn Fern</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>Chamaedorea elegans</t>
+          <t>Platycerium bifurcatum</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect light or light shade; protect the fine leaflets from strong direct sun.</t>
+          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>Check below the surface before watering; keep lightly moist in growth but never leave the shared planter waterlogged.</t>
+          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>Keep warm, remove only fully brown fronds at the base and feed monthly at low strength in spring and summer.</t>
+          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>Evergreen fine-textured fronds provide the display throughout the year; growth is slowest in winter.</t>
+          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · Shared Pot · Arrowhead Vine</t>
+          <t>House · Sitting Room · Shared Pot · Spider Plant</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Arrowhead Vine — assumed</t>
+          <t>Spider Plant ‘Vittatum’ — assumed</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Chlorophytum comosum ‘Vittatum’</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect light; keep the leaves out of strong direct sun through the glass.</t>
+          <t>Bright indirect light is ideal; it tolerates lower light but direct hot sun can scorch the striped leaves.</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>Keep lightly moist during active growth, allowing the surface to begin drying; water more sparingly in winter.</t>
+          <t>Allow the compost surface to begin drying, then water thoroughly and let the shared container drain fully.</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>Guide or trim lengthening stems in spring, feed during active growth and wear gloves if pruning because the sap is irritating.</t>
+          <t>Trim only spent stems or badly damaged leaves, feed lightly during active growth and root the hanging plantlets if wanted.</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>Evergreen juvenile arrow-shaped leaves become more divided as stems mature; indoor flowering is uncommon.</t>
+          <t>Evergreen striped foliage and hanging plantlets are the year-round display; growth slows in winter.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Sitting Room · Shared Pot · Parlour Palm</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Cleopatra'</t>
+          <t>Parlour Palm — assumed</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
+          <t>Chamaedorea elegans</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Bright indirect light or light shade; protect the fine leaflets from strong direct sun.</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
+          <t>Check below the surface before watering; keep lightly moist in growth but never leave the shared planter waterlogged.</t>
         </is>
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
+          <t>Keep warm, remove only fully brown fronds at the base and feed monthly at low strength in spring and summer.</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
+          <t>Evergreen fine-textured fronds provide the display throughout the year; growth is slowest in winter.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Sitting Room · Shared Pot · Arrowhead Vine</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Antarctica'</t>
+          <t>Arrowhead Vine — assumed</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Antarctica'</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Bright indirect light; keep the leaves out of strong direct sun through the glass.</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
+          <t>Keep lightly moist during active growth, allowing the surface to begin drying; water more sparingly in winter.</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
+          <t>Guide or trim lengthening stems in spring, feed during active growth and wear gloves if pruning because the sap is irritating.</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
+          <t>Evergreen juvenile arrow-shaped leaves become more divided as stems mature; indoor flowering is uncommon.</t>
         </is>
       </c>
     </row>
@@ -6969,148 +6969,222 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
+          <t>Skimmia 'Cleopatra'</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>Viola cornuta 'Rocky Purple Picotee'</t>
+          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost evenly moist but well drained.</t>
+          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
         </is>
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
+          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>Purple flowers with pale picotee margins through the cool season.</t>
+          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Viburnum 'Lisarose'</t>
+          <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Viburnum tinus 'Lisarose'</t>
+          <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+          <t>Keep the shared compost evenly moist but well drained.</t>
         </is>
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+          <t>Purple flowers with pale picotee margins through the cool season.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum tinus 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
           <t>Viburnum Pot</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus Spirit</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus 'Anvi' (Spirit)</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>Sun or partial shade, with shelter from cold drying winds.</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>Keep evenly moist but well drained while establishing; check the pot through dry and windy weather.</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>Prune only after flowering if needed. Refresh the top compost in spring and protect the container during prolonged severe cold.</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>Pink buds open to lightly fragrant creamy-white flowers from late winter into spring, followed by blue-black ornamental berries.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G180"/>
+  <autoFilter ref="A1:G182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Combine Nicola's shared houseplants into one planter record
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant Guide" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$L$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$L$187</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plant Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13419,71 +13419,75 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · Shared Pot · Spider Plant</t>
+          <t>House · Sitting Room · Nicola’s Mixed Planter</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Spider Plant ‘Vittatum’ — assumed</t>
+          <t>Nicola’s Mixed Planter — identities assumed</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Chlorophytum comosum ‘Vittatum’</t>
+          <t>Chlorophytum · Chamaedorea · Syngonium</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect. Tolerates lower light; hot direct sun can mark the foliage</t>
+          <t>Bright indirect. Filter strong sitting-room window sun and keep smaller companions visible</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Let the surface begin drying, then soak and drain the shared pot</t>
+          <t>Moderate · shared root ball. Test below the surface in several places, water evenly when needed and drain fully</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>Keep the window light filtered: Bright indirect light maintains clean variegation. The sitting-room window is useful light, but move the planter back or filter the glass if strong direct sun begins bleaching or scorching the leaves.
-Water the shared root ball, then drain: Use the compost, not a calendar, to decide. Test below the surface in several places because the large clump can hide dry pockets. Water thoroughly only when the surface is beginning to dry and never leave runoff in the outer container.
-Choose which plantlets to keep: The long runners are healthy propagation growth. Root wanted plantlets in small pots while still attached, then cut the connecting stem. Remove spent flowering stems only when no more plantlets are wanted.
-Review crowding in spring: Three vigorous species are sharing one root space. If water runs straight through, the centre stays dry or growth weakens, slide out the root ball in spring and decide whether to divide the Spider Plant or separate the three species.</t>
+          <t>Give all three plants filtered light: Bright indirect light suits the shared display. Filter harsh glass sun and guide the dominant Spider Plant leaves away from the palm’s small crown and the vine. Rotate the pot for balanced growth.
+Water the pot once, checking several pockets: One container needs one moisture decision. Test around the palm, vine and pot edge. Water evenly when the surface begins to dry, keeping the active-growth root ball lightly moist but never saturated. Empty runoff and lengthen watering intervals in winter.
+Trim each component appropriately: Keep the mixed canopy open without cutting healthy palm growth. Root or remove selected Spider Plant plantlets; remove only fully brown palm fronds at their bases. Guide or shorten long Arrowhead Vine stems in spring, wearing gloves and keeping cuttings out of reach.
+Review crowding during spring growth: The Spider Plant’s fleshy roots can crowd its companions. If water races through, dry pockets persist or smaller plants weaken, inspect the shared root ball in spring. Divide or separate only if congestion warrants it; feed modestly during active growth using the product instructions.</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>Spring: Look for fresh striped leaves and plantlets, feed lightly and check whether the Spider Plant's fleshy roots are displacing its two pot companions.
-Summer: Keep the striped rosette in filtered light, water the shared pot only after checking depth and trim brown tips without cutting healthy green tissue.
-Autumn: Remove spent plantlet stems and stop feeding as growth slows, noting whether its vigorous roots are making separation necessary.
-Winter: Maximise gentle light for the white stripe, water sparingly and keep leaf tips away from the sitting-room radiator.</t>
+          <t>Spring: Inspect the shared root ball for crowding as fresh growth starts; manage Spider Plant plantlets, retain green palm fronds and guide or shorten vine stems with gloves.
+Summer: Filter strong window sun, test moisture near all three plants, rotate the planter and inspect palm fronds and vine leaf undersides for pests.
+Autumn: Stop routine feeding as growth slows, remove spent runners and fully brown foliage, and keep the complete planter clear of cold window draughts.
+Winter: Give the whole pot gentle daylight and steady warmth; water less often after checking depth and keep leaves away from radiator air.</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>The dominant cascading plant in Nicola’s mixed gift pot is a Spider Plant. Its creamy central leaf stripe, green margins and long runners carrying young plantlets closely fit Chlorophytum comosum ‘Vittatum’; the cultivar remains visibly assumed because no label has been retained.</t>
+          <t>One large sitting-room pot gifted by Nicola, Katie’s mum. An arching Spider Plant ‘Vittatum’, upright Parlour Palm and smaller Arrowhead Vine grow together in the same container. These photo-based identities remain assumed without retained labels; the planter is recorded and watered as one unit.</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>Habit: Arching clump. Long striped leaves form a dense fountain over the shared planter
-Light: Bright indirect. Tolerates lower light; hot direct sun can mark the foliage
-Water: Moderate. Let the surface begin drying, then soak and drain the shared pot
-Plantlets: Many runners. Young plants can be rooted while attached or removed once rooted
-Identity: ‘Vittatum’ assumed. Central creamy stripes and especially long arching leaves support the best fit
-Pet safety: Non-toxic listed. ASPCA listing for Chlorophytum
-Care priority: Keep runners off the smaller companions. Trim or pot selected spider plantlets before the vigorous arching growth shades the shared planter's palm and vine.</t>
+          <t>Contents: Three plants · one pot. Assumed Spider Plant ‘Vittatum’, Parlour Palm and Arrowhead Vine
+Light: Bright indirect. Filter strong sitting-room window sun and keep smaller companions visible
+Water: Moderate · shared root ball. Test below the surface in several places, water evenly when needed and drain fully
+Temperature: Warm indoor position. Protect the shared display from cold glass, draughts and radiator heat
+Habit: Arching, upright and climbing. Spider Plant runners surround fine palm fronds and juvenile arrow-shaped vine leaves
+Safety: Contains an irritant vine. Treat the whole shared planter as harmful if eaten because of the Arrowhead Vine
+Care priority: Check the whole mixed planter. Test moisture near all three plants, keep the palm and vine clear of Spider Plant runners and handle the Arrowhead Vine with gloves.</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>Species confidence is high from the diagnostic runners and striped leaves. The central stripe and long arching habit make ‘Vittatum’ the leading cultivar, but it remains assumed without a retained label. Nicola, Katie’s mum, gave the complete three-plant pot to Oak Lodge.</t>
+          <t>Nicola, Katie’s mum, gave the complete planter to Oak Lodge. Central creamy stripes and runners support Chlorophytum comosum ‘Vittatum’; fine pinnate fronds support Chamaedorea elegans; arrow-shaped leaves and a climbing stem support Syngonium podophyllum. All component identities remain visibly assumed. Brad confirmed in October 2026 that they should be recorded together as one pot.</t>
         </is>
       </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
-          <t>https://www.rhs.org.uk/plants/67933/chlorophytum-comosum-vittatum-v/details
-https://www.rhs.org.uk/plants/spider-plants/growing-guide
-https://www.aspca.org/pet-care/aspca-poison-control/toxic-and-non-toxic-plants/chlorophytum</t>
+          <t>https://www.rhs.org.uk/plants/spider-plants/growing-guide
+https://www.rhs.org.uk/plants/67933/chlorophytum-comosum-vittatum-v/details
+https://www.rhs.org.uk/plants/chamaedorea/growing-guide
+https://www.rhs.org.uk/plants/17899/syngonium-podophyllum/details
+https://www.aspca.org/pet-care/aspca-poison-control/toxic-and-non-toxic-plants/chlorophytum
+https://www.aspca.org/pet-care/aspca-poison-control/toxic-and-non-toxic-plants/chamaedorea
+https://www.aspca.org/pet-care/aspca-poison-control/toxic-and-non-toxic-plants/arrow-head-vine</t>
         </is>
       </c>
       <c r="L176" s="2" t="inlineStr">
@@ -13495,188 +13499,37 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · Shared Pot · Parlour Palm</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>Parlour Palm — assumed</t>
+          <t>Skimmia 'Cleopatra'</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>Chamaedorea elegans</t>
+          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>Indirect or light shade. Forest-understorey foliage scorches in strong direct sun</t>
+          <t>Partial or full shade. Shelter from strong sun and drying wind</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Moist but free-draining in growth; less water in winter</t>
+          <t>Avoid a dry root ball. Shade and reliable drainage matter; yellowing alone does not mean iron deficiency.</t>
         </is>
       </c>
       <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>Shelter the fine fronds from sun: Bright indirect light or light shade suits this understorey palm. Direct summer sun through the sitting-room glass can scorch or bleach the leaflets. Rotate the shared planter periodically for balanced light.
-Avoid permanent wetness: The palm likes regular moisture with air around its roots. Check the shared root ball before watering, soak evenly when it has begun to dry and empty all runoff. Reduce the frequency as winter growth slows.
-Keep old fronds until fully brown: Remove only finished growth at the base. Do not cut green leaflet tips into a tidy shape. Remove a frond cleanly at its base only after it has become fully brown.
-Feed and repot gently: Slow growth needs modest feeding and infrequent disturbance. Apply a balanced liquid feed monthly during spring and summer. Review the whole mixed root ball in spring if crowding or uneven drying becomes a problem.</t>
-        </is>
-      </c>
-      <c r="G177" s="2" t="inlineStr">
-        <is>
-          <t>Spring: Watch for a new palm spear before beginning weak feed, and inspect the shared planter for crowding around the Palm's fine roots.
-Summer: Keep the fronds in bright filtered light, rotate the shared pot for even growth and check for spider mite in dry weather.
-Autumn: Stop feeding, remove only fully brown fronds at the base and protect the delicate leaflets from cold window draughts.
-Winter: Maintain steady room temperature and modest humidity, watering only after the shared compost has partly dried below the surface.</t>
-        </is>
-      </c>
-      <c r="H177" s="2" t="inlineStr">
-        <is>
-          <t>The upright plant rising through Nicola’s mixed gift pot is a Parlour Palm. Its slender clustered stems and compact pinnate fronds with many narrow leaflets strongly fit Chamaedorea elegans; the photo-based identification remains visibly assumed until a label is found.</t>
-        </is>
-      </c>
-      <c r="I177" s="2" t="inlineStr">
-        <is>
-          <t>Indoor size: Usually 30–60cm. Slow growing indoors, though old plants can eventually become larger
-Light: Indirect or light shade. Forest-understorey foliage scorches in strong direct sun
-Water: Moderate. Moist but free-draining in growth; less water in winter
-Temperature: Warm room. RHS recommends roughly 10–27°C, with stronger growth around 20–27°C
-Identity: Chamaedorea elegans. Fine pinnate fronds and slender stems support a high-confidence photo identification
-Pet safety: Non-toxic listed. ASPCA listing for Chamaedorea elegans
-Care priority: Expose the palm's small crown to light. Guide Spider Plant leaves away from the palm and inspect its fine fronds for mites in dry room air.</t>
-        </is>
-      </c>
-      <c r="J177" s="2" t="inlineStr">
-        <is>
-          <t>The fine pinnate fronds, numerous narrow leaflets and slender clustered stems make Parlour palm a high-confidence best fit, retained as assumed without a label. Nicola, Katie’s mum, gave the complete three-plant pot to Oak Lodge.</t>
-        </is>
-      </c>
-      <c r="K177" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rhs.org.uk/plants/chamaedorea/growing-guide
-https://www.rhs.org.uk/plants/29185/chamaedorea-elegans/details
-https://www.aspca.org/pet-care/aspca-poison-control/toxic-and-non-toxic-plants/chamaedorea</t>
-        </is>
-      </c>
-      <c r="L177" s="2" t="inlineStr">
-        <is>
-          <t>house-sitting-mixed-parlour-palm</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>House · Sitting Room · Shared Pot · Arrowhead Vine</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>Arrowhead Vine — assumed</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>Bright indirect. Green forms tolerate partial shade; strong direct sun can scorch</t>
-        </is>
-      </c>
-      <c r="E178" s="2" t="inlineStr">
-        <is>
-          <t>Lightly moist. Water freely in active growth, more sparingly in winter, always with drainage</t>
-        </is>
-      </c>
-      <c r="F178" s="2" t="inlineStr">
-        <is>
-          <t>Keep it bright without harsh sun: Filtered window light maintains compact leafy growth. The larger Spider Plant may shade it heavily, so watch new growth for stretching while also preventing direct sun through the glass.
-Balance moisture across the shared pot: This vine prefers slightly steadier moisture than its companions. Test the compost around the vine as well as at the pot edge. Water the whole container when needed, drain fully and reduce watering in winter.
-Guide or shorten long stems: Arrowhead Vine naturally becomes a climber. Add a small support or trim leggy stems in spring. Wear gloves, keep sap away from eyes and wash tools and hands after pruning.
-Keep away from pets and children: Every part should be treated as harmful if chewed. Place the shared planter and any cuttings out of reach. Seek veterinary or medical advice promptly after suspected ingestion or significant sap exposure.</t>
-        </is>
-      </c>
-      <c r="G178" s="2" t="inlineStr">
-        <is>
-          <t>Spring: Pinch the Arrowhead Vine above a node to encourage a compact shoot and begin light feeding only when new arrow-shaped leaves open.
-Summer: Guide or trim the fastest vine so it does not climb through the Palm, and check undersides of tender leaves for pests.
-Autumn: Stop feeding, remove yellow leaves at their petioles and decide whether the increasingly vining habit still suits the shared planter.
-Winter: Give the Arrowhead Vine bright indirect light, protect it from cold glass and allow the upper shared compost to dry slightly between checks.</t>
-        </is>
-      </c>
-      <c r="H178" s="2" t="inlineStr">
-        <is>
-          <t>The smaller arrow-leaved plant tucked beneath the Spider Plant is an Arrowhead Vine. Its juvenile sagittate leaves, pale midrib and climbing stem strongly support Syngonium podophyllum. No cultivar can be resolved from these photographs, and the species remains visibly assumed until labelled.</t>
-        </is>
-      </c>
-      <c r="I178" s="2" t="inlineStr">
-        <is>
-          <t>Habit: Climbing vine. Compact while young, then lengthens and can be guided or allowed to trail
-Light: Bright indirect. Green forms tolerate partial shade; strong direct sun can scorch
-Water: Lightly moist. Water freely in active growth, more sparingly in winter, always with drainage
-Temperature: Above 15°C. RHS rates it H1A for warm indoor conditions
-Identity: Species assumed. Juvenile arrow-shaped leaves and climbing stem support Syngonium podophyllum
-Safety: Oxalate irritant. Harmful if eaten and irritating to skin and eyes
-Care priority: Keep the vine accessible and out of reach. Trim climbing stems before they disappear through the palm, and keep this irritant plant away from pets and children.</t>
-        </is>
-      </c>
-      <c r="J178" s="2" t="inlineStr">
-        <is>
-          <t>Juvenile arrow-shaped leaves, pale venation and a climbing stem make Syngonium podophyllum a high-confidence best fit, but the species remains assumed and no cultivar is claimed. Nicola, Katie’s mum, gave the complete three-plant pot to Oak Lodge.</t>
-        </is>
-      </c>
-      <c r="K178" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rhs.org.uk/plants/17899/syngonium-podophyllum/details
-https://www.aspca.org/pet-care/aspca-poison-control/toxic-and-non-toxic-plants/arrow-head-vine</t>
-        </is>
-      </c>
-      <c r="L178" s="2" t="inlineStr">
-        <is>
-          <t>house-sitting-mixed-arrowhead-vine</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia Pot</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia 'Cleopatra'</t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
-        </is>
-      </c>
-      <c r="D179" s="2" t="inlineStr">
-        <is>
-          <t>Partial or full shade. Shelter from strong sun and drying wind</t>
-        </is>
-      </c>
-      <c r="E179" s="2" t="inlineStr">
-        <is>
-          <t>Avoid a dry root ball. Shade and reliable drainage matter; yellowing alone does not mean iron deficiency.</t>
-        </is>
-      </c>
-      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>Shade the Skimmia's roots: Keep moisture steady without standing water. Skimmias do not require ericaceous compost. Check exposure, dryness and drainage before trying to correct yellow leaves with iron or acidifying products.
 Preserve flowers and possible berries: Prune only wayward or damaged shoots, usually in spring. Heavy clipping removes flower buds. Female forms generally need a nearby male to set fruit; two female plants do not supply that pollen.
 Check pollination before expecting berries: For this Oak Lodge specimen Cleopatra shares the pot with Antarctica; do not assume the second Skimmia supplies compatible male flowers.</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>Spring: Use rainwater where practical, feed with an ericaceous product after flowering and leave pollinated flower clusters intact for berries.
 Summer: Keep evenly moist in warm weather, checking beneath the ivy before watering.
@@ -13684,12 +13537,12 @@
 Winter: Keep drainage open and protect the decorative container during prolonged hard frost.</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>Cleopatra forms one of the evergreen centres of the Skimmia Pot, with glossy foliage and fragrant pale spring flowers. This female selection can carry red berries when compatible pollen is available; sharing a pot with another female does not provide it. Shade, an evenly moist root ball and drainage matter more than acidity: Skimmias do not require ericaceous compost.</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr">
         <is>
           <t>Size: About 0.5–1m. Compact rounded shrub suited to a large pot
 Position: Partial or full shade. Shelter from strong sun and drying wind
@@ -13701,57 +13554,57 @@
 Care priority: Check pollination before expecting berries. Cleopatra shares the pot with Antarctica; do not assume the second Skimmia supplies compatible male flowers.</t>
         </is>
       </c>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>The supplied garden record confirms Cleopatra; the registered cultivar epithet ‘Snep24’ and female berry-bearing habit come from the cultivar reference.</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/skimmia/growing-guide
 https://plantariumgroendirekt.nl/nieuwigheden-en/skimmia-japonica-snep24-cleopatra/?lang=en</t>
         </is>
       </c>
-      <c r="L179" s="2" t="inlineStr">
+      <c r="L177" s="2" t="inlineStr">
         <is>
           <t>lobeliapot-skimmia-cleopatra</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>Skimmia Pot</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>Partial shade. Sheltered shade reduces yellowing caused by hot dry exposure.</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>Avoid a dry root ball. Shade and reliable drainage matter; yellowing alone does not mean iron deficiency.</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>Shade the Skimmia's roots: Keep moisture steady without standing water. Skimmias do not require ericaceous compost. Check exposure, dryness and drainage before trying to correct yellow leaves with iron or acidifying products.
 Preserve flowers and possible berries: Prune only wayward or damaged shoots, usually in spring. Heavy clipping removes flower buds. Female forms generally need a nearby male to set fruit; two female plants do not supply that pollen.
 Record Antarctica's flowers and fruit: For this Oak Lodge specimen Retain its separate label and observe the berry colour rather than copying Cleopatra's red-fruit description.</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>Spring: Enjoy the fragrant flower clusters, remove frost-burned leaves individually and top-dress with fresh peat-free compost without covering the stem bases.
 Summer: Keep this evergreen pot evenly moist in hot weather and sheltered from harsh midday sun; do not shear off the developing berry clusters.
@@ -13759,12 +13612,12 @@
 Winter: Move the pot out of drying wind, raise it on feet and water only on frost-free days when the compost below the surface is genuinely dry.</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>Antarctica is the second labelled Skimmia in the blue pot, sharing its root space with Cleopatra and three Rocky Purple Picotee Violas. Its compact evergreen framework gives year-round structure, while the spring flowers and any later fruit should be recorded separately from Cleopatra. Protect the root ball from drying and avoid assuming that pale foliage needs acidifying treatment.</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr">
         <is>
           <t>Size: Compact shrub. Cultivar dimensions need verification; pot size is not a permanent height limit.
 Position: Partial shade. Sheltered shade reduces yellowing caused by hot dry exposure.
@@ -13776,57 +13629,57 @@
 Care priority: Record Antarctica's flowers and fruit. Retain its separate label and observe the berry colour rather than copying Cleopatra's red-fruit description.</t>
         </is>
       </c>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>The supplied September update and photographs record this plant's identity and position.</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/skimmia/growing-guide
 https://www.rhs.org.uk/plants/364299/skimmia-japonica-antarctica/details</t>
         </is>
       </c>
-      <c r="L180" s="2" t="inlineStr">
+      <c r="L178" s="2" t="inlineStr">
         <is>
           <t>lobeliapot-skimmia-antarctica</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>Skimmia Pot</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>Sun to partial shade. Keep the low flowers open to light beneath the two Skimmias.</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>Moist, with free drainage. Small Viola and pansy roots dry quickly; cool, saturated compost can rot their crowns.</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>Remove flowers and seed capsules: Pinch each spent stem back to a leaf joint. Clear rain-damaged blooms promptly to limit grey mould. A light feed during growth helps sustain flowers in a container.
 Let cool weather set the pace: Expect pauses during hard frost or summer heat. Trim stretched stems to leafy growth if the crown is sound. Give light shade in hot weather and avoid burying small crowns under fallen leaves.
 Check all three low crowns: For this Oak Lodge specimen Keep the three Rocky Purple Picotee plants clear of fallen Skimmia leaves and inspect each small root plug.</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>Spring: Deadhead back to a leaf joint, trim winter-scorched edges and give a light feed once fresh buds begin to move.
 Summer: Keep spent flowers and seed capsules removed; if heat stops flowering, shade the pot in the afternoon and expect a cooler-weather recovery.
@@ -13834,12 +13687,12 @@
 Winter: Pick off collapsed petals before botrytis spreads and protect the small root ball from alternating waterlogging and hard frost.</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>Three Rocky Purple Picotee Violas form a low purple-and-pale-edged flowering layer beneath the two Skimmias. Their cool-season display can pause in hard frost or summer heat. Each little crown needs light, airflow and reliable moisture, with spent flower stems and seed capsules removed before the shared pot becomes crowded with decaying petals.</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr">
         <is>
           <t>Size: 15–25cm. Typical bedding-Viola height; three separate plants are recorded in this pot.
 Position: Sun to partial shade. Keep the low flowers open to light beneath the two Skimmias.
@@ -13851,56 +13704,56 @@
 Care priority: Check all three low crowns. Keep the three Rocky Purple Picotee plants clear of fallen Skimmia leaves and inspect each small root plug.</t>
         </is>
       </c>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>The supplied September update and photographs record this plant's identity and position.</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/education-learning/children-young-people/family-activities/grow-it/pansy</t>
         </is>
       </c>
-      <c r="L181" s="2" t="inlineStr">
+      <c r="L179" s="2" t="inlineStr">
         <is>
           <t>lobeliapot-viola-rocky-purple-picotee</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>Bed 2/3 Wall Pot</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Viburnum ‘Lisarose’ — label confirmed</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus ‘Lisarose’</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>Sun to shade. Shelter from cold drying winds</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>Check the pot all year. Evergreen Viburnum still loses moisture in winter; water only when the root ball needs it and is unfrozen.</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>Prune after the winter flowers: Shorten only outgrowing branches after the spring display. Viburnum tinus develops the next flowers on its existing framework. Heavy late-summer or autumn trimming sacrifices buds; removing spent heads also reduces subsequent berries.
 Allow for a shrub-sized root system: Top-dress in spring and repot when roots fill the container. Use a stable, drained loam-based container mix. Check leaf undersides and new shoots for Viburnum beetle damage rather than assuming every hole is drought stress.
 Allow Lisarose room above the Vinca: For this Oak Lodge specimen Keep the wall pot's ivy-like trailer off the Viburnum base and plan greater root room as the shrub grows.</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>Spring: Let flowering finish before any shaping, top-dress lightly and inspect for viburnum beetle damage.
 Summer: Water the shared pot deeply during drought and take semi-ripe cuttings only if propagation is wanted.
@@ -13908,12 +13761,12 @@
 Winter: Enjoy the flower clusters and protect the container from prolonged freezing while keeping drainage open.</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>‘Lisarose’ is the upright evergreen centre of the new pot between Beds 2 and 3. Deep brick-red buds intensify as temperatures fall, then open to pink-and-white flower clusters from midwinter into spring, followed by dark blue ornamental berries. Its eventual shrub size means the current shared pot is an establishment home rather than unlimited permanent root space.</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr">
         <is>
           <t>Size: Potentially 2.5–4m. Large dense shrub if planted in open ground
 Position: Sun to shade. Shelter from cold drying winds
@@ -13925,56 +13778,56 @@
 Care priority: Allow Lisarose room above the Vinca. Keep the wall pot's ivy-like trailer off the Viburnum base and plan greater root room as the shrub grows.</t>
         </is>
       </c>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>The photographed label explicitly reads Viburnum Lisarose. This supersedes the earlier unresolved garden record.</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/302763/viburnum-tinus-lisarose-pbr-laurustinus-lisarose/details</t>
         </is>
       </c>
-      <c r="L182" s="2" t="inlineStr">
+      <c r="L180" s="2" t="inlineStr">
         <is>
           <t>bed23wallpot-viburnum-lisarose</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>Bed 2/3 Wall Pot</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Vinca minor ‘Illumination’ — label confirmed</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>Vinca minor ‘Illumination’</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>Sun to shade. Bright shade retains colour without scorching</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>Moderate; avoid prolonged drying. Vinca tolerates some dry shade once established, but trailing plants in pots still depend on the container's moisture.</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>Keep Vinca runners within bounds: Shorten trails that root into neighbouring planting. Remove unwanted rooted pieces completely. Trim after the main spring flowers, retaining leafy growth for the next display.
 Remove green reversions: Cut all-green shoots back to their point of origin. Variegated forms can be overtaken by vigorous green growth. Give enough light for leaf colour without letting the shallow roots bake.
 Keep the additional Vinca on the wall: For this Oak Lodge specimen Trim rooted runners before this second Illumination leaves its shared wall pot or smothers Lisarose.</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>Spring: Trim winter damage, guide fresh runners and enjoy the violet flowers.
 Summer: Shorten stems that reach unwanted soil and keep them clear of the Viburnum crown.
@@ -13982,12 +13835,12 @@
 Winter: Keep drainage holes open and water only when the compost is genuinely dry.</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>This is a second, additional Vinca minor ‘Illumination’, planted to trail over the Bed 2/3 dividing wall while the original remains in the Bed 5 big pot. Broad gold leaf centres edged narrowly in green provide year-round colour, with violet-blue flowers from spring into autumn. Rooting runners make it effective but require deliberate containment.</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr">
         <is>
           <t>Size: 10–15cm high. Trailing stems can extend 60–90cm
 Position: Sun to shade. Bright shade retains colour without scorching
@@ -13999,56 +13852,56 @@
 Care priority: Keep the additional Vinca on the wall. Trim rooted runners before this second Illumination leaves its shared wall pot or smothers Lisarose.</t>
         </is>
       </c>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>The retained name and distinctive gold-centred foliage confirm this additional ‘Illumination’ specimen. This supersedes the earlier unresolved garden record.</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/161486/vinca-minor-illumination-v/details</t>
         </is>
       </c>
-      <c r="L183" s="2" t="inlineStr">
+      <c r="L181" s="2" t="inlineStr">
         <is>
           <t>bed23wallpot-vinca-minor-illumination</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>Viburnum Pot</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus Spirit — label confirmed</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus ‘Anvi’ (Spirit)</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>Sun or partial shade. Shelter from cold drying winds</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>Check the pot all year. Evergreen Viburnum still loses moisture in winter; water only when the root ball needs it and is unfrozen.</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>Prune after the winter flowers: Shorten only outgrowing branches after the spring display. Viburnum tinus develops the next flowers on its existing framework. Heavy late-summer or autumn trimming sacrifices buds; removing spent heads also reduces subsequent berries.
 Allow for a shrub-sized root system: Top-dress in spring and repot when roots fill the container. Use a stable, drained loam-based container mix. Check leaf undersides and new shoots for Viburnum beetle damage rather than assuming every hole is drought stress.
 Inspect the separate Spirit pot: For this Oak Lodge specimen Check drainage and root crowding in Spirit's own glazed pot rather than assuming it matches the shared Lisarose container.</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>Spring: Let flowering finish, then prune only if needed and refresh the top layer of compost.
 Summer: Water deeply through drought, feed lightly and inspect for viburnum beetle or whitefly.
@@ -14056,12 +13909,12 @@
 Winter: Keep the pot drained, protect it from prolonged hard freezes and enjoy the developing flower clusters.</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus Spirit (‘Anvi’) fills the new glazed pot at the foot of the steps with glossy evergreen foliage and a long winter display. Pink buds open to lightly fragrant creamy-white clusters from late winter into spring, followed by blue-black ornamental berries. The shrub can reach about two metres, so root room, feeding and winter protection around the pot matter as it matures.</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr">
         <is>
           <t>Size: Up to about 2m. Compact rounded shrub with a similar spread
 Position: Sun or partial shade. Shelter from cold drying winds
@@ -14073,56 +13926,56 @@
 Care priority: Inspect the separate Spirit pot. Check drainage and root crowding in Spirit's own glazed pot rather than assuming it matches the shared Lisarose container.</t>
         </is>
       </c>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>The photographed nursery label reads Viburnum tinus Spirit; ‘Anvi’ is its accepted cultivar epithet. This supersedes the earlier unresolved garden record.</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/196958/viburnum-tinus-spirit-%28anvipbr%29/details</t>
         </is>
       </c>
-      <c r="L184" s="2" t="inlineStr">
+      <c r="L182" s="2" t="inlineStr">
         <is>
           <t>viburnumpot-viburnum-tinus-spirit</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>House · Sitting Room · Rhipsalis (species to confirm)</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Rhipsalis (species to confirm)</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>Rhipsalis sp.</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>Bright indirect. Protect the trails from harsh window sun.</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>Surface drying. Drain after watering; avoid sustained dryness.</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>Check the hanging pot: Feel the compost before watering. Soak when its surface dries, then drain away from furniture.
 Protect its long trails: Keep stems clear of the stairs. The purple star records the hanging point; check that walking past does not snag growth.
 Give filtered light: Avoid harsh direct sunshine. Observe pale or puckered stems and adjust light or moisture after checking the roots.</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>Spring: Watch for fresh branching and increase checks as growth resumes.
 Summer: Check the exposed hanging root ball during warm spells.
@@ -14130,12 +13983,12 @@
 Winter: Keep the hanging cactus warm and water less often.</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>The new Rhipsalis hangs beside the sitting-room stair opening, its slender green stems falling in a long curtain. Brad supplied the genus name; species remains unresolved. Care follows mistletoe-cactus guidance provisionally, with observation of this specimen taking priority.</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr">
         <is>
           <t>Habit: Trailing stems. The October photograph shows a hanging specimen.
 Light: Bright indirect. Protect the trails from harsh window sun.
@@ -14145,57 +13998,57 @@
 Care priority: Keep the hanging root ball accessible. Check moisture in the hanging pot itself and keep the long trails clear of the split-level stair opening.</t>
         </is>
       </c>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>Genus supplied by Brad; no species or cultivar claimed from the photograph.</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr">
         <is>
           <t>https://plants.ces.ncsu.edu/plants/rhipsalis-baccifera/
 https://www.rhs.org.uk/plants/14483/rhipsalis-baccifera/details</t>
         </is>
       </c>
-      <c r="L185" s="2" t="inlineStr">
+      <c r="L183" s="2" t="inlineStr">
         <is>
           <t>house-sitting-rhipsalis</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>House · Sitting Room / stair opening · Dracaena Bicolour Touffe</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Dracaena Bicolour Touffe</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>Dracaena marginata Bicolor type — assumed</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>Indirect light. Shelter at the stair opening.</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>Upper compost drying. Avoid stagnant runoff.</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>Water the inner pot: Allow the upper compost to dry. Drain thoroughly and use rainwater where possible.
 Keep leaves out of traffic: Check the green-star stair position. Rotate only enough to maintain balanced growth without obstructing the passage.
 Clean and inspect the tufts: Wipe dust from strap-shaped leaves. Inspect for pests; avoid repeatedly wetting an already damp root ball.</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>Spring: Watch the two crowns for new leaves and restart modest feeding.
 Summer: Protect narrow leaves from strong glass-filtered sun and draughts.
@@ -14203,12 +14056,12 @@
 Winter: Keep the stair-side plant warm and reduce watering further.</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>Brad’s “Dracena Bicolour Touffe” is recorded as Dracaena Bicolour Touffe. The two narrow-leaved tufts beside the split-level stairs fit a marginata-type dragon tree. The formal Bicolor cultivar relationship remains assumed without a retained passport.</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr">
         <is>
           <t>Habit: Upright leafy tufts. Two crowns are visible in the small pot.
 Light: Indirect light. Shelter at the stair opening.
@@ -14218,57 +14071,57 @@
 Care priority: Protect the two stair-side tufts. Keep leaves clear of passing feet; verify natural light and drain the small inner pot after watering.</t>
         </is>
       </c>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>Name supplied by Brad; Dracaena marginata Bicolor type is a qualified photo fit.</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/dracaena/how-to-grow-dracaena
 https://www.rhs.org.uk/plants/dracaena</t>
         </is>
       </c>
-      <c r="L186" s="2" t="inlineStr">
+      <c r="L184" s="2" t="inlineStr">
         <is>
           <t>house-sitting-dracaena-bicolour</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>House · Bedroom-wing landing · Crassula 'Hottentot'</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Crassula 'Hottentot'</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>Crassula rupestris subsp. marnieriana type</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>Very bright. The lamp is part of the display; assess actual daylight.</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>Dry between drinks. Use the inner-pot weight and compost together.</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>Empty the decorative pot: Water only after drying. Soak the inner pot separately and let runoff finish before replacing it.
 Assess daylight at the shelf: Give the succulent strong natural light. Introduce direct sun gradually; watch stretching at the orange-star position.
 Keep the leaf strings sound: Handle trailing growth gently. Remove only damaged portions and inspect tightly stacked leaves for mealybugs.</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>Spring: Resume moderate watering once the leaf strings extend.
 Summer: Maintain bright light and allow drying between soakings.
@@ -14276,12 +14129,12 @@
 Winter: Water the landing succulent sparingly and keep it warm.</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>Crassula ‘Hottentot’ spills over the landing shelf in dense bead-like strings of fleshy paired leaves. The supplied commercial name is retained, while its botanical placement follows the marnieriana worm-plant type provisionally. The orange star marks the shelf beside the lamp.</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr">
         <is>
           <t>Habit: Pendant leafy strings. Long trails spill from the decorative pot.
 Light: Very bright. The lamp is part of the display; assess actual daylight.
@@ -14291,57 +14144,57 @@
 Care priority: Check natural light on the landing shelf. The table lamp does not establish adequate daylight; monitor stretching and let the succulent compost dry between drinks.</t>
         </is>
       </c>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>Commercial name supplied by Brad; marnieriana botanical fit remains provisional.</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/4749/crassula-rupestris-subsp-marnieriana/details
 https://powo.science.kew.org/taxon/urn%3Alsid%3Aipni.org%3Anames%3A878790-1</t>
         </is>
       </c>
-      <c r="L187" s="2" t="inlineStr">
+      <c r="L185" s="2" t="inlineStr">
         <is>
           <t>house-landing-crassula-hottentot</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>House · Kitchen / Dining · Philodendron (species to confirm)</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Philodendron (species to confirm)</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>Philodendron sp.</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>Bright indirect. Protect leaves at the kitchen window.</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>Upper compost drying. Use airy compost and free drainage.</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>Check the kitchen root ball: Water after surface drying. Drain the orange pot fully before returning it to the window.
 Leave space for new leaves: Protect tender foliage from sun scorch. Observe growth before deciding whether this particular plant needs a climbing support.
 Handle with care: Keep it out of reach. Wear gloves when cutting and clean tools after contact with sap.</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>Spring: Record the next leaves to help resolve identity and habit.
 Summer: Check the small kitchen pot more often during warm weather.
@@ -14349,12 +14202,12 @@
 Winter: Keep the Philodendron away from cold window glass.</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>The birthday photograph records a small Philodendron in an orange pot. Brad’s red star places it at the kitchen / dining window. Species, cultivar and eventual climbing or upright habit remain unresolved, so this portrait uses genus guidance and keeps those questions visible.</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr">
         <is>
           <t>Light: Bright indirect. Protect leaves at the kitchen window.
 Water: Upper compost drying. Use airy compost and free drainage.
@@ -14364,56 +14217,56 @@
 Care priority: Record the next kitchen-window leaves. Retain species uncertainty, inspect new growth before choosing a support and keep the orange pot fully drained.</t>
         </is>
       </c>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>Philodendron genus supplied by Brad; species and cultivar unresolved.</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/plants/philodendron/growing-guide</t>
         </is>
       </c>
-      <c r="L188" s="2" t="inlineStr">
+      <c r="L186" s="2" t="inlineStr">
         <is>
           <t>house-kitchen-philodendron</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>House · Bedroom-wing landing · Zamioculcas</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Zamioculcas</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>Zamioculcas zamiifolia — assumed</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>Indirect; shade tolerated. Lower light lengthens drying time.</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>Root ball drying. Check deeply before the next drink.</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>Let the root ball dry: Check below the surface. Water thoroughly only after drying and let all runoff escape.
 Protect the landing leaves: Keep upright stalks away from traffic. The blue star sits beside the stair opening; avoid scraping leaflets when passing.
 Inspect glossy leaflets: Wipe dust gently. Look for scale on stalks and leaf undersides; feed sparingly during active growth.</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>Spring: Watch for new upright shoots and check whether the pot is congested.
 Summer: Allow full drying even while the landing is warm.
@@ -14421,12 +14274,12 @@
 Winter: Keep the rhizomes dry between occasional winter drinks.</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>Zamioculcas stands beside the console on the bedroom-wing landing, with glossy leaflets on upright fleshy stalks. Its photograph strongly supports Zamioculcas zamiifolia, retained as assumed without a label. The blue star records the position beside Bedroom 3.</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr">
         <is>
           <t>Habit: Upright glossy leaves. Fleshy stalks rise from underground rhizomes.
 Light: Indirect; shade tolerated. Lower light lengthens drying time.
@@ -14436,24 +14289,24 @@
 Care priority: Let the fleshy rhizomes dry between drinks. Check deep compost at the blue-star landing position before watering; avoid trapping runoff beneath the nursery pot.</t>
         </is>
       </c>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>Supplied genus and glossy pinnate leaves strongly support Z. zamiifolia; retained as assumed.</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr">
         <is>
           <t>https://plants.ces.ncsu.edu/plants/zamioculcas-zamiifolia/</t>
         </is>
       </c>
-      <c r="L189" s="2" t="inlineStr">
+      <c r="L187" s="2" t="inlineStr">
         <is>
           <t>house-landing-zamioculcas</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L189"/>
+  <autoFilter ref="A1:L187"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace Bed 1 basket rescues with Pernettya and Solanum
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -1485,69 +1485,68 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia (cultivar to confirm)</t>
+          <t>Pernettya Pink (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia hybrid</t>
+          <t>Gaultheria mucronata — pink-fruited form</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Sheltered partial shade. Back Bed 1 beneath the Japanese Maple</t>
+          <t>Sun to partial shade. Monitor shade beneath the Maple; record whether this pocket gets sufficient light.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Moist during active Bed 1 growth. The former basket root ball needs establishment water, but the sheltered crown must not sit in cold wet soil.</t>
+          <t>Even moisture at roots. Check this new planting separately from its established neighbours.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Wait for spring buds before pruning: Cut winter-damaged stems back only after living growth is visible. The cultivar and hardiness are unresolved. Preserve useful low buds and pinch young shoots only if a bushier border framework is needed.
-Support the arching flowers: Keep Fuchsia stems clear of the fern and Skimmia crowns. Deadhead during the mild season, feed lightly only while growing and photograph open flowers from the side and front for later identification.
-Support the moved Bed 1 stems: For this Oak Lodge specimen Arrange the arching Fuchsia clear of the fern and Skimmia crowns while its new root system establishes.</t>
+          <t>Check the acidic pocket: Test soil pH if it is unknown. Use an acidic root environment for Pernettya; if this bed is unsuitable, an ericaceous container is a practical alternative.
+Keep berry-bearing growth: Avoid a hard autumn trim. Remove damaged shoots and control unwanted suckers. Keep the small plant clear of expanding Hosta leaves.
+Check future pollination: Existing berries do not guarantee next year’s crop. Female Gaultheria mucronata normally needs a compatible male nearby; confirm the selection before buying a partner.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Spring: Wait for live buds before cutting winter-damaged stems, then pinch young shoots only if a bushier Bed 1 framework is needed.
-Summer: Water the new root area during dry spells, feed lightly while flowering and support arching stems away from the fern crown.
-Autumn: Stop feeding, record a fully open flower for identification and mulch lightly without covering the stem base.
-Winter: Protect the newly planted crown until its hardiness is known and wait for spring buds before declaring bare upper stems dead.</t>
+          <t>Spring: Check new shoots and remove unwanted suckers without disturbing the Pernettya root ball.
+Summer: Watch the little bell flowers and check moisture beneath the Maple as its canopy fills.
+Autumn: Enjoy the photographed pink fruit and keep bark away from the Pernettya stem base.
+Winter: Check that the evergreen Pernettya root ball drains freely and does not dry during prolonged dry weather.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>The former Hanging Basket 3 Fuchsia now grows beneath the Japanese Maple in Back Bed 1, where its arching stems carry pendant bicolour flowers among the newly moved fern and Skimmia. The trailing habit is secure, but colour and cultivar are not recorded, so final size and winter hardiness remain deliberately unresolved.</t>
+          <t>Pernettya Pink brings pale pink and stronger pink berries to the cleared pocket beside the Buddha beneath the Japanese Maple. Brad supplied the name; the photograph fits a pink-fruited Gaultheria mucronata, but does not establish a named cultivar such as Pink Pearl. It replaces part of the space left by the discarded September Fuchsia and fern.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Size: 20–60cm high. Arching stems may spread beyond the former basket scale
-Position: Sheltered partial shade. Back Bed 1 beneath the Japanese Maple
-Soil: Moist and well-drained. Humus-rich bed soil with reliable drainage
-Hardiness: To confirm. The cultivar is unresolved; protect the crown during its first winter in the bed
-Main feature: Pendant bicolour flowers. Arching flowers among the shaded Bed 1 planting
-Identity: Fuchsia cultivar. Cultivar and exact flower colours are not recorded
-Water: Moist during active Bed 1 growth. The former basket root ball needs establishment water, but the sheltered crown must not sit in cold wet soil.
-Care priority: Support the moved Bed 1 stems. Arrange the arching Fuchsia clear of the fern and Skimmia crowns while its new root system establishes.</t>
+          <t>Identity: Pink-fruited Gaultheria. Pernettya is an older name; Pink does not identify a particular cultivar.
+Size: About 0.5–1m. Cultivar size remains unresolved; record this specimen’s spread.
+Position: Sun to partial shade. Monitor shade beneath the Maple; record whether this pocket gets sufficient light.
+Soil: Acidic, moist and drained. Check pH before relying on the bed for long-term ericaceous growth.
+Hardiness: Hardy species. Pink-form cultivar rating not confirmed.
+Flower: White bells · late spring / early summer. The pink display is fruit, not flowers.
+Water: Even moisture at roots. Check this new planting separately from its established neighbours.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia identity and its move from Hanging Basket 3 to Back Bed 1 are secure from the garden record; cultivar is unresolved.</t>
+          <t>Name supplied by Brad, October 2026. Photos support the plant group and berry colour; cultivar confirmation remains pending.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rhs.org.uk/plants/84426/fuchsia-mrs-popple/details</t>
+          <t>https://www.rhs.org.uk/plants/67076/gaultheria-mucronata-pink-pearl-f/details</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>baskets-trailing-fuchsia</t>
+          <t>bed1-pernettya-pink</t>
         </is>
       </c>
     </row>
@@ -1559,69 +1558,69 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Fern (cultivar to confirm)</t>
+          <t>Solanum 'Jupiter' (name supplied)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Fern — cultivar to confirm</t>
+          <t>Solanum pseudocapsicum 'Jupiter' — supplied trade name</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Sheltered shade to partial shade. Filtered light protects soft fronds while its exact shade preference remains unresolved.</t>
+          <t>Sunny, sheltered position. Monitor shade beneath the Maple; record whether this pocket gets sufficient light.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Even moisture in sheltered soil. The moved fern needs a cool root area beneath the Maple but its crown must not remain saturated.</t>
+          <t>Even moisture at roots. Check this new planting separately from its established neighbours.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Protect the moved frond crown: Remove only dead fronds at their base and clear fallen Maple leaves. Do not shear the plant or feed it for flowers. Brown spore patches can be normal; keep the crown exposed to air as it establishes in Bed 1.
-Use new growth for identification: Photograph croziers, scales and mature frond undersides. Until the species is resolved, protect the new planting during hard frost rather than assuming the hardiness of a known garden fern.
-Keep a frond for identification: For this Oak Lodge specimen Photograph the moved Bed 1 fern's underside before removing old fronds; its winter requirements are still unresolved.</t>
+          <t>Plan for frost: Arrange frost-free accommodation if keeping Jupiter. It is recorded as planted in Bed 1, but is a seasonal outdoor display unless suitable frost-free accommodation becomes available.
+Water its own root ball: Feel the soil before adding water. The nursery root ball can dry while surrounding bark and soil look damp. Keep drainage open and reduce watering in cool conditions.
+Handle fruit safely: Keep children and pets away from the berries. All parts are poisonous. Wear gloves, collect fallen berries and never treat the fruit as food.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Spring: Remove only brown fronds at their base and photograph new croziers, scales and mature frond undersides to narrow the identification.
-Summer: Use the Maple canopy as shelter from hot midday sun, maintaining even moisture while keeping the crown open to air.
-Autumn: Clear fallen leaves before they smother the crown and record whether the fronds remain evergreen as temperatures fall.
-Winter: Because the species is unconfirmed, add light protection during hard frost and keep the sheltered crown just moist rather than saturated.</t>
+          <t>Spring: If Jupiter has survived frost-free, inspect living growth before any light shaping.
+Summer: Give Jupiter good light during flowering; inspect leaves for aphids and mites.
+Autumn: Enjoy Jupiter’s orange and red fruit; arrange frost-free conditions before damaging cold.
+Winter: If retained frost-free, give Jupiter bright light and reduced watering; assess outdoor frost damage before deciding its future.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>The unidentified fern moved from Hanging Basket 3 into the sheltered soil beneath the Japanese Maple in Back Bed 1. Its divided green fronds now form a low foliage layer beside the moved Fuchsia and Skimmia. Brown spore patches can be normal, but species and hardiness remain unresolved, so preserve diagnostic photographs and use cautious first-winter protection.</t>
+          <t>Solanum Jupiter adds bright green, yellow, orange and red fruit in front of the Hosta in the cleared Bed 1 pocket. The supplied name and photograph fit the ornamental winter-cherry group, Solanum pseudocapsicum. Jupiter is recorded as Brad’s supplied trade name, with a label still needed for confirmation. This is a tender seasonal planting.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Size: Species not yet identified. Measure the fronds and record their form; basket size is not a mature plant dimension.
-Position: Sheltered shade to partial shade. Filtered light protects soft fronds while its exact shade preference remains unresolved.
-Soil: Humus-rich, moist and free-draining soil. Keep the frond-producing crown above the compost and prevent the small root plug drying hard.
-Hardiness: Unresolved; protect from frost. An unidentified fern must not inherit the hardy Dryopteris rating.
-Main feature: Divided green fronds. Fronds are the display: this fern produces spores, not flowers.
-Identity: Fern (cultivar to confirm). Name retained from the supplied garden record
-Water: Even moisture in sheltered soil. The moved fern needs a cool root area beneath the Maple but its crown must not remain saturated.
-Care priority: Keep a frond for identification. Photograph the moved Bed 1 fern's underside before removing old fronds; its winter requirements are still unresolved.</t>
+          <t>Identity: Jupiter · name supplied. Brad supplied Jupiter; no label photograph confirms the name.
+Size: Species can reach about 0.9m. Nursery selections may stay smaller; record the height of this plant.
+Position: Sunny, sheltered position. Monitor shade beneath the Maple; record whether this pocket gets sufficient light.
+Soil: Moist, well-drained loam. Water the small root ball without keeping the planting hole saturated.
+Hardiness: Tender; frost-free winter. An outdoor wall or fleece cannot guarantee frost-free conditions.
+Flower: White stars · summer. The coloured balls are ornamental fruit, not edible tomatoes.
+Water: Even moisture at roots. Check this new planting separately from its established neighbours.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>The supplied September update and photographs record this plant's identity and position.</t>
+          <t>Name supplied by Brad, October 2026. Photos support the plant group and berry colour; cultivar confirmation remains pending.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rhs.org.uk/plants/types/ferns/growing-guide</t>
+          <t>https://plants.ces.ncsu.edu/plants/solanum-pseudocapsicum/
+https://pages.nxtbook.com/syngenta/FloriProServices/Pot_Plants_2016_EX/offline/FloriProServices_Pot_Plants_2016_EX.pdf</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>baskets-fern-unidentified</t>
+          <t>bed1-solanum-jupiter</t>
         </is>
       </c>
     </row>

</xml_diff>